<commit_message>
fiestapp v2 - remove secrets and scratch scripts
</commit_message>
<xml_diff>
--- a/public/assets/plantilla_invitados.xlsx
+++ b/public/assets/plantilla_invitados.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>PLANTILLA JANO'S - REGISTRO DE INVITADOS</t>
   </si>
@@ -22,18 +22,12 @@
     <t>Apellido</t>
   </si>
   <si>
-    <t>Numero de Mesa</t>
-  </si>
-  <si>
     <t>Juan</t>
   </si>
   <si>
     <t>Pérez</t>
   </si>
   <si>
-    <t>Mesa 1</t>
-  </si>
-  <si>
     <t>María</t>
   </si>
   <si>
@@ -46,16 +40,10 @@
     <t>Maza</t>
   </si>
   <si>
-    <t>Mesa 2</t>
-  </si>
-  <si>
     <t>Ana</t>
   </si>
   <si>
     <t>Gómez</t>
-  </si>
-  <si>
-    <t>Mesa 3</t>
   </si>
 </sst>
 </file>
@@ -512,78 +500,61 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="1" max="2" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="45" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" ht="45" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
     </row>
-    <row r="2" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="2" t="s">
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
         <v>3</v>
       </c>
+      <c r="B3" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="3" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="3" t="s">
+    <row r="4" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+    <row r="5" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>6</v>
-      </c>
     </row>
-    <row r="5" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+    <row r="6" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B6" s="4" t="s">
         <v>10</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>14</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
mayor fixes and pdates
</commit_message>
<xml_diff>
--- a/public/assets/plantilla_invitados.xlsx
+++ b/public/assets/plantilla_invitados.xlsx
@@ -4,16 +4,19 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Invitados" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Plantilla Invitados" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
-  <si>
-    <t>PLANTILLA JANO'S - REGISTRO DE INVITADOS</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+  <si>
+    <t>miFiestAPP  •  REGISTRO DE INVITADOS</t>
+  </si>
+  <si>
+    <t>Completá nombres, apellidos y teléfonos de tus invitados</t>
   </si>
   <si>
     <t>Nombre</t>
@@ -22,35 +25,53 @@
     <t>Apellido</t>
   </si>
   <si>
+    <t>Teléfono (Opcional)</t>
+  </si>
+  <si>
     <t>Juan</t>
   </si>
   <si>
     <t>Pérez</t>
   </si>
   <si>
+    <t>11 1234 5678</t>
+  </si>
+  <si>
     <t>María</t>
   </si>
   <si>
     <t>López</t>
   </si>
   <si>
+    <t>11 8765 4321</t>
+  </si>
+  <si>
     <t>Esteban</t>
   </si>
   <si>
     <t>Maza</t>
   </si>
   <si>
+    <t>11 9999 8888</t>
+  </si>
+  <si>
     <t>Ana</t>
   </si>
   <si>
     <t>Gómez</t>
+  </si>
+  <si>
+    <t>11 5555 4444</t>
+  </si>
+  <si>
+    <t>© 2026 miFiestAPP  •  Digitalizá Tu Fiesta  •  www.mifiestapp.com.ar</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -61,8 +82,13 @@
     <font>
       <b/>
       <color rgb="FFD4AF37"/>
-      <family val="2"/>
-      <sz val="13"/>
+      <sz val="12"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFF3E5AB"/>
+      <sz val="9"/>
       <name val="Segoe UI"/>
     </font>
     <font>
@@ -72,12 +98,18 @@
       <name val="Segoe UI"/>
     </font>
     <font>
-      <color rgb="FF333333"/>
+      <color rgb="FFF0F0F5"/>
       <sz val="10"/>
       <name val="Segoe UI"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FFD4AF37"/>
+      <sz val="9"/>
+      <name val="Segoe UI"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -86,22 +118,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1A1A1A"/>
+        <fgColor rgb="FF111113"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF2A2A2A"/>
+        <fgColor rgb="FF1F1F24"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
+        <fgColor rgb="FF1F1A0A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF9F9F9"/>
+        <fgColor rgb="FF161619"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1E1E23"/>
       </patternFill>
     </fill>
   </fills>
@@ -115,13 +152,13 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF444444"/>
+        <color rgb="FF3A2F0F"/>
       </left>
       <right style="thin">
-        <color rgb="FF444444"/>
+        <color rgb="FF3A2F0F"/>
       </right>
       <top style="thin">
-        <color rgb="FF444444"/>
+        <color rgb="FF3A2F0F"/>
       </top>
       <bottom style="medium">
         <color rgb="FFD4AF37"/>
@@ -129,17 +166,13 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FFDCDCDC"/>
-      </left>
+      <left/>
       <right style="thin">
-        <color rgb="FFDCDCDC"/>
+        <color rgb="FF2A2A30"/>
       </right>
-      <top style="thin">
-        <color rgb="FFDCDCDC"/>
-      </top>
+      <top/>
       <bottom style="thin">
-        <color rgb="FFDCDCDC"/>
+        <color rgb="FF2A2A30"/>
       </bottom>
       <diagonal/>
     </border>
@@ -147,18 +180,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -500,61 +539,95 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="2" width="35" customWidth="1"/>
+    <col min="1" max="3" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="45" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" ht="38" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
-    </row>
-    <row r="2" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C1" s="1"/>
+    </row>
+    <row r="2" ht="24" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+    </row>
+    <row r="3" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" ht="26" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+    <row r="5" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B5" s="4" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="5" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="3" t="s">
+    </row>
+    <row r="6" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="6" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>10</v>
       </c>
     </row>
+    <row r="7" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="10" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" s="6"/>
+      <c r="C10" s="6"/>
+    </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
+  <mergeCells count="3">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A10:C10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>